<commit_message>
Los tiempos de la plantilla se escriben en segundos
Escribir el TMO como mm:ss obligaba a dejar la celda en formato de texto,
porque con formato de hora Excel lo convertía en hora del día. El precio
era que la fórmula de cumplimiento comparaba letra por letra: «1200» le
ganaba a «700», porque el 1 va antes que el 7, y un agente fuera de meta
aparecía cumpliendo.

Ahora TMO y TMR se escriben en segundos enteros, con celdas numéricas y
una comparación normal. Las metas quedan en 700 y 30 segundos. El portal
los sigue mostrando como minutos y segundos, que es como se leen bien.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UGm45zgMxnFLLEQHs5AtTV
</commit_message>
<xml_diff>
--- a/plantilla/Plantilla_Resultados.xlsx
+++ b/plantilla/Plantilla_Resultados.xlsx
@@ -206,10 +206,10 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,7 +218,7 @@
     <xf numFmtId="164" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -699,7 +699,7 @@
       <c r="B18" s="2" t="inlineStr">
         <is>
           <t>· Porcentajes: escribe 95% o 0,95. La celda ya viene con formato de porcentaje.
-· Tiempos (TMO, TMR): escribe minutos y segundos, como 3:05. Esas celdas vienen en formato de texto a propósito, para que Excel no te las convierta en hora del día.
+· Tiempos (TMO, TMR): escribe SEGUNDOS enteros, como 700. No escribas 11:40. El portal los muestra convertidos a minutos y segundos, pero la comparación con la meta tiene que ser entre números.
 · Cantidades: números enteros, sin puntos de miles.
 · Si un agente no tiene medición en un indicador, deja la celda vacía. El portal lo marca como no cumple y se nota a simple vista.
 · La columna CUMPLIMIENTO se calcula sola. Es para que tú lo veas aquí; el portal no la usa para decidir, él vuelve a comparar resultado contra meta.</t>
@@ -1026,23 +1026,19 @@
         <v/>
       </c>
       <c r="O3" s="18" t="n"/>
-      <c r="P3" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P3" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q3" s="17">
-        <f>IF(O3="","",IF(IFERROR(TIMEVALUE(O3),99)&lt;=IFERROR(TIMEVALUE(P3),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O3="","",IF(O3&lt;=P3,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R3" s="18" t="n"/>
-      <c r="S3" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S3" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T3" s="17">
-        <f>IF(R3="","",IF(IFERROR(TIMEVALUE(R3),99)&lt;=IFERROR(TIMEVALUE(S3),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R3="","",IF(R3&lt;=S3,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U3" s="15" t="n"/>
@@ -1100,23 +1096,19 @@
         <v/>
       </c>
       <c r="O4" s="18" t="n"/>
-      <c r="P4" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P4" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q4" s="17">
-        <f>IF(O4="","",IF(IFERROR(TIMEVALUE(O4),99)&lt;=IFERROR(TIMEVALUE(P4),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O4="","",IF(O4&lt;=P4,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R4" s="18" t="n"/>
-      <c r="S4" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S4" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T4" s="17">
-        <f>IF(R4="","",IF(IFERROR(TIMEVALUE(R4),99)&lt;=IFERROR(TIMEVALUE(S4),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R4="","",IF(R4&lt;=S4,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U4" s="15" t="n"/>
@@ -1174,23 +1166,19 @@
         <v/>
       </c>
       <c r="O5" s="18" t="n"/>
-      <c r="P5" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P5" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q5" s="17">
-        <f>IF(O5="","",IF(IFERROR(TIMEVALUE(O5),99)&lt;=IFERROR(TIMEVALUE(P5),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O5="","",IF(O5&lt;=P5,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R5" s="18" t="n"/>
-      <c r="S5" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S5" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T5" s="17">
-        <f>IF(R5="","",IF(IFERROR(TIMEVALUE(R5),99)&lt;=IFERROR(TIMEVALUE(S5),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R5="","",IF(R5&lt;=S5,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U5" s="15" t="n"/>
@@ -1248,23 +1236,19 @@
         <v/>
       </c>
       <c r="O6" s="18" t="n"/>
-      <c r="P6" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P6" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q6" s="17">
-        <f>IF(O6="","",IF(IFERROR(TIMEVALUE(O6),99)&lt;=IFERROR(TIMEVALUE(P6),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O6="","",IF(O6&lt;=P6,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R6" s="18" t="n"/>
-      <c r="S6" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S6" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T6" s="17">
-        <f>IF(R6="","",IF(IFERROR(TIMEVALUE(R6),99)&lt;=IFERROR(TIMEVALUE(S6),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R6="","",IF(R6&lt;=S6,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U6" s="15" t="n"/>
@@ -1322,23 +1306,19 @@
         <v/>
       </c>
       <c r="O7" s="18" t="n"/>
-      <c r="P7" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P7" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q7" s="17">
-        <f>IF(O7="","",IF(IFERROR(TIMEVALUE(O7),99)&lt;=IFERROR(TIMEVALUE(P7),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O7="","",IF(O7&lt;=P7,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R7" s="18" t="n"/>
-      <c r="S7" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S7" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T7" s="17">
-        <f>IF(R7="","",IF(IFERROR(TIMEVALUE(R7),99)&lt;=IFERROR(TIMEVALUE(S7),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R7="","",IF(R7&lt;=S7,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U7" s="15" t="n"/>
@@ -1396,23 +1376,19 @@
         <v/>
       </c>
       <c r="O8" s="18" t="n"/>
-      <c r="P8" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P8" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q8" s="17">
-        <f>IF(O8="","",IF(IFERROR(TIMEVALUE(O8),99)&lt;=IFERROR(TIMEVALUE(P8),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O8="","",IF(O8&lt;=P8,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R8" s="18" t="n"/>
-      <c r="S8" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S8" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T8" s="17">
-        <f>IF(R8="","",IF(IFERROR(TIMEVALUE(R8),99)&lt;=IFERROR(TIMEVALUE(S8),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R8="","",IF(R8&lt;=S8,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U8" s="15" t="n"/>
@@ -1470,23 +1446,19 @@
         <v/>
       </c>
       <c r="O9" s="18" t="n"/>
-      <c r="P9" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P9" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q9" s="17">
-        <f>IF(O9="","",IF(IFERROR(TIMEVALUE(O9),99)&lt;=IFERROR(TIMEVALUE(P9),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O9="","",IF(O9&lt;=P9,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R9" s="18" t="n"/>
-      <c r="S9" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S9" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T9" s="17">
-        <f>IF(R9="","",IF(IFERROR(TIMEVALUE(R9),99)&lt;=IFERROR(TIMEVALUE(S9),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R9="","",IF(R9&lt;=S9,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U9" s="15" t="n"/>
@@ -1544,23 +1516,19 @@
         <v/>
       </c>
       <c r="O10" s="18" t="n"/>
-      <c r="P10" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P10" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q10" s="17">
-        <f>IF(O10="","",IF(IFERROR(TIMEVALUE(O10),99)&lt;=IFERROR(TIMEVALUE(P10),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O10="","",IF(O10&lt;=P10,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R10" s="18" t="n"/>
-      <c r="S10" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S10" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T10" s="17">
-        <f>IF(R10="","",IF(IFERROR(TIMEVALUE(R10),99)&lt;=IFERROR(TIMEVALUE(S10),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R10="","",IF(R10&lt;=S10,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U10" s="15" t="n"/>
@@ -1618,23 +1586,19 @@
         <v/>
       </c>
       <c r="O11" s="18" t="n"/>
-      <c r="P11" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P11" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q11" s="17">
-        <f>IF(O11="","",IF(IFERROR(TIMEVALUE(O11),99)&lt;=IFERROR(TIMEVALUE(P11),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O11="","",IF(O11&lt;=P11,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R11" s="18" t="n"/>
-      <c r="S11" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S11" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T11" s="17">
-        <f>IF(R11="","",IF(IFERROR(TIMEVALUE(R11),99)&lt;=IFERROR(TIMEVALUE(S11),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R11="","",IF(R11&lt;=S11,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U11" s="15" t="n"/>
@@ -1692,23 +1656,19 @@
         <v/>
       </c>
       <c r="O12" s="18" t="n"/>
-      <c r="P12" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P12" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q12" s="17">
-        <f>IF(O12="","",IF(IFERROR(TIMEVALUE(O12),99)&lt;=IFERROR(TIMEVALUE(P12),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O12="","",IF(O12&lt;=P12,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R12" s="18" t="n"/>
-      <c r="S12" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S12" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T12" s="17">
-        <f>IF(R12="","",IF(IFERROR(TIMEVALUE(R12),99)&lt;=IFERROR(TIMEVALUE(S12),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R12="","",IF(R12&lt;=S12,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U12" s="15" t="n"/>
@@ -1766,23 +1726,19 @@
         <v/>
       </c>
       <c r="O13" s="18" t="n"/>
-      <c r="P13" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P13" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q13" s="17">
-        <f>IF(O13="","",IF(IFERROR(TIMEVALUE(O13),99)&lt;=IFERROR(TIMEVALUE(P13),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O13="","",IF(O13&lt;=P13,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R13" s="18" t="n"/>
-      <c r="S13" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S13" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T13" s="17">
-        <f>IF(R13="","",IF(IFERROR(TIMEVALUE(R13),99)&lt;=IFERROR(TIMEVALUE(S13),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R13="","",IF(R13&lt;=S13,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U13" s="15" t="n"/>
@@ -1840,23 +1796,19 @@
         <v/>
       </c>
       <c r="O14" s="18" t="n"/>
-      <c r="P14" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P14" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q14" s="17">
-        <f>IF(O14="","",IF(IFERROR(TIMEVALUE(O14),99)&lt;=IFERROR(TIMEVALUE(P14),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O14="","",IF(O14&lt;=P14,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R14" s="18" t="n"/>
-      <c r="S14" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S14" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T14" s="17">
-        <f>IF(R14="","",IF(IFERROR(TIMEVALUE(R14),99)&lt;=IFERROR(TIMEVALUE(S14),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R14="","",IF(R14&lt;=S14,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U14" s="15" t="n"/>
@@ -1914,23 +1866,19 @@
         <v/>
       </c>
       <c r="O15" s="18" t="n"/>
-      <c r="P15" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P15" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q15" s="17">
-        <f>IF(O15="","",IF(IFERROR(TIMEVALUE(O15),99)&lt;=IFERROR(TIMEVALUE(P15),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O15="","",IF(O15&lt;=P15,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R15" s="18" t="n"/>
-      <c r="S15" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S15" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T15" s="17">
-        <f>IF(R15="","",IF(IFERROR(TIMEVALUE(R15),99)&lt;=IFERROR(TIMEVALUE(S15),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R15="","",IF(R15&lt;=S15,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U15" s="15" t="n"/>
@@ -1988,23 +1936,19 @@
         <v/>
       </c>
       <c r="O16" s="18" t="n"/>
-      <c r="P16" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P16" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q16" s="17">
-        <f>IF(O16="","",IF(IFERROR(TIMEVALUE(O16),99)&lt;=IFERROR(TIMEVALUE(P16),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O16="","",IF(O16&lt;=P16,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R16" s="18" t="n"/>
-      <c r="S16" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S16" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T16" s="17">
-        <f>IF(R16="","",IF(IFERROR(TIMEVALUE(R16),99)&lt;=IFERROR(TIMEVALUE(S16),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R16="","",IF(R16&lt;=S16,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U16" s="15" t="n"/>
@@ -2062,23 +2006,19 @@
         <v/>
       </c>
       <c r="O17" s="18" t="n"/>
-      <c r="P17" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P17" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q17" s="17">
-        <f>IF(O17="","",IF(IFERROR(TIMEVALUE(O17),99)&lt;=IFERROR(TIMEVALUE(P17),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O17="","",IF(O17&lt;=P17,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R17" s="18" t="n"/>
-      <c r="S17" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S17" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T17" s="17">
-        <f>IF(R17="","",IF(IFERROR(TIMEVALUE(R17),99)&lt;=IFERROR(TIMEVALUE(S17),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R17="","",IF(R17&lt;=S17,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U17" s="15" t="n"/>
@@ -2136,23 +2076,19 @@
         <v/>
       </c>
       <c r="O18" s="18" t="n"/>
-      <c r="P18" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P18" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q18" s="17">
-        <f>IF(O18="","",IF(IFERROR(TIMEVALUE(O18),99)&lt;=IFERROR(TIMEVALUE(P18),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O18="","",IF(O18&lt;=P18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R18" s="18" t="n"/>
-      <c r="S18" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S18" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T18" s="17">
-        <f>IF(R18="","",IF(IFERROR(TIMEVALUE(R18),99)&lt;=IFERROR(TIMEVALUE(S18),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R18="","",IF(R18&lt;=S18,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U18" s="15" t="n"/>
@@ -2452,23 +2388,19 @@
         <v/>
       </c>
       <c r="O3" s="18" t="n"/>
-      <c r="P3" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P3" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q3" s="17">
-        <f>IF(O3="","",IF(IFERROR(TIMEVALUE(O3),99)&lt;=IFERROR(TIMEVALUE(P3),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O3="","",IF(O3&lt;=P3,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R3" s="18" t="n"/>
-      <c r="S3" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S3" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T3" s="17">
-        <f>IF(R3="","",IF(IFERROR(TIMEVALUE(R3),99)&lt;=IFERROR(TIMEVALUE(S3),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R3="","",IF(R3&lt;=S3,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U3" s="15" t="n"/>
@@ -2526,23 +2458,19 @@
         <v/>
       </c>
       <c r="O4" s="18" t="n"/>
-      <c r="P4" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P4" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q4" s="17">
-        <f>IF(O4="","",IF(IFERROR(TIMEVALUE(O4),99)&lt;=IFERROR(TIMEVALUE(P4),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O4="","",IF(O4&lt;=P4,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R4" s="18" t="n"/>
-      <c r="S4" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S4" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T4" s="17">
-        <f>IF(R4="","",IF(IFERROR(TIMEVALUE(R4),99)&lt;=IFERROR(TIMEVALUE(S4),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R4="","",IF(R4&lt;=S4,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U4" s="15" t="n"/>
@@ -2600,23 +2528,19 @@
         <v/>
       </c>
       <c r="O5" s="18" t="n"/>
-      <c r="P5" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P5" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q5" s="17">
-        <f>IF(O5="","",IF(IFERROR(TIMEVALUE(O5),99)&lt;=IFERROR(TIMEVALUE(P5),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O5="","",IF(O5&lt;=P5,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R5" s="18" t="n"/>
-      <c r="S5" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S5" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T5" s="17">
-        <f>IF(R5="","",IF(IFERROR(TIMEVALUE(R5),99)&lt;=IFERROR(TIMEVALUE(S5),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R5="","",IF(R5&lt;=S5,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U5" s="15" t="n"/>
@@ -2674,23 +2598,19 @@
         <v/>
       </c>
       <c r="O6" s="18" t="n"/>
-      <c r="P6" s="22" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P6" s="22" t="n">
+        <v>700</v>
       </c>
       <c r="Q6" s="17">
-        <f>IF(O6="","",IF(IFERROR(TIMEVALUE(O6),99)&lt;=IFERROR(TIMEVALUE(P6),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O6="","",IF(O6&lt;=P6,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R6" s="18" t="n"/>
-      <c r="S6" s="22" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S6" s="22" t="n">
+        <v>30</v>
       </c>
       <c r="T6" s="17">
-        <f>IF(R6="","",IF(IFERROR(TIMEVALUE(R6),99)&lt;=IFERROR(TIMEVALUE(S6),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R6="","",IF(R6&lt;=S6,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U6" s="15" t="n"/>
@@ -2748,23 +2668,19 @@
         <v/>
       </c>
       <c r="O7" s="18" t="n"/>
-      <c r="P7" s="19" t="inlineStr">
-        <is>
-          <t>3:00</t>
-        </is>
+      <c r="P7" s="19" t="n">
+        <v>700</v>
       </c>
       <c r="Q7" s="17">
-        <f>IF(O7="","",IF(IFERROR(TIMEVALUE(O7),99)&lt;=IFERROR(TIMEVALUE(P7),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(O7="","",IF(O7&lt;=P7,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="R7" s="18" t="n"/>
-      <c r="S7" s="19" t="inlineStr">
-        <is>
-          <t>0:30</t>
-        </is>
+      <c r="S7" s="19" t="n">
+        <v>30</v>
       </c>
       <c r="T7" s="17">
-        <f>IF(R7="","",IF(IFERROR(TIMEVALUE(R7),99)&lt;=IFERROR(TIMEVALUE(S7),0),"CUMPLE","NO CUMPLE"))</f>
+        <f>IF(R7="","",IF(R7&lt;=S7,"CUMPLE","NO CUMPLE"))</f>
         <v/>
       </c>
       <c r="U7" s="15" t="n"/>

</xml_diff>